<commit_message>
EMS-1: initial commit of event management system
</commit_message>
<xml_diff>
--- a/registrations.xlsx
+++ b/registrations.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,31 +462,391 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>mandar mavalankar</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>mandarmavalankar@gmail.com</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>7588271179</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>STABILIA Robotics Workshop 2K26</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Robitics analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>mandar mavalankar</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>mandarmavalankar@gmail.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>7588271179</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>STABILIA Robotics Workshop 2K26</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Robitics analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>28</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>mandar mavalankar</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>mandarmavalankar@gmail.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>7588271179</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Kalakruti 2K26</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Poster Making</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>29</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>mandar mavalankar</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>mandarmavalankar@gmail.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>7588271179</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>STABILIA Robotics Workshop 2K26</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Robitics analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>30</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>sakshi kudtarkar</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>atharvk4406@gmail.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>7588271179</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Sports Day 2K26</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Football</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>32</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>Aniruddha Takke</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>aniruddha4406@gmail.com</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>7588271179</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>atharvk4406@gmail.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>7588271179</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Kalakruti 2K26</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Painting</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>33</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>mandar mavalankar</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>atharvkudtarkar4406@okhdfcbank</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>7588271179</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>STABILIA Robotics Workshop 2K26</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Robitics analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>34</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>mandar mavalankar</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>atharvkudtarkar4406@okhdfcbank</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>7588271179</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>STABILIA Robotics Workshop 2K26</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Robitics analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>35</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>mandar mavalankar</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>atharvkudtarkar4406@okhdfcbank</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>7588271179</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>STABILIA Robotics Workshop 2K26</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Robitics analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>36</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>mandar mavalankar</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>atharvkudtarkar4406@okhdfcbank</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>7588271179</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>STABILIA Robotics Workshop 2K26</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Robitics analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>37</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Pratik</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>atharvkudtarkar4406@gmail.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>7588271179</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Kalakruti 2K26</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Rangoli</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>40</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Shrikant</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>atharvkudtarkar4406@gmail.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>7588271179</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>UTOPIA 2K26</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Dance</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>49</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Pratik</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>atharvkudtarkar4406@gmail.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>7588271179</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Kalakruti 2K26</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Rangoli</t>
         </is>
       </c>
     </row>

</xml_diff>